<commit_message>
new file for Napoli sim
</commit_message>
<xml_diff>
--- a/collections/Scorecards_e_assegnazione/eureca_input_final_blank.xlsx
+++ b/collections/Scorecards_e_assegnazione/eureca_input_final_blank.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unipdit.sharepoint.com/sites/BETALAB/Documenti condivisi/UBEM PD/URBEM_Scorecards/v6/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pratenr82256\Desktop\Nest_UBEM\collections\Scorecards_e_assegnazione\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_B437E5379A9C801789F76FA0F5174A4C7FFC1CCB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4366A581-EE09-49C7-8942-907F6EB02D5E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15CD99AA-AB4F-444A-923B-4C50EF009618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1890" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="810" yWindow="-120" windowWidth="28110" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Envelopes" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8436" uniqueCount="2385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8446" uniqueCount="2395">
   <si>
     <t>id</t>
   </si>
@@ -7179,6 +7179,36 @@
   </si>
   <si>
     <t>RES_SINGLE_1992-2005_E_VAL_window</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>e</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>laz</t>
+  </si>
+  <si>
+    <t>lig</t>
+  </si>
+  <si>
+    <t>lomb</t>
+  </si>
+  <si>
+    <t>sic</t>
+  </si>
+  <si>
+    <t>vall</t>
   </si>
 </sst>
 </file>
@@ -7202,12 +7232,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -7237,11 +7273,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7546,13 +7583,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I329"/>
+  <dimension ref="A1:R329"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="31.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7578,7 +7615,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -7607,7 +7644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -7635,8 +7672,23 @@
       <c r="I3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="N3" t="s">
+        <v>2390</v>
+      </c>
+      <c r="O3" t="s">
+        <v>2391</v>
+      </c>
+      <c r="P3" t="s">
+        <v>2392</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>2393</v>
+      </c>
+      <c r="R3" t="s">
+        <v>2394</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -7664,8 +7716,14 @@
       <c r="I4">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="M4" t="s">
+        <v>2387</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -7693,8 +7751,14 @@
       <c r="I5">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="M5" t="s">
+        <v>2385</v>
+      </c>
+      <c r="O5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -7722,8 +7786,17 @@
       <c r="I6">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="M6" t="s">
+        <v>2386</v>
+      </c>
+      <c r="N6" s="2">
+        <v>2</v>
+      </c>
+      <c r="O6">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -7751,8 +7824,20 @@
       <c r="I7">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="M7" t="s">
+        <v>2388</v>
+      </c>
+      <c r="O7">
+        <v>20</v>
+      </c>
+      <c r="P7">
+        <v>4</v>
+      </c>
+      <c r="R7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -7780,8 +7865,14 @@
       <c r="I8">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="M8" t="s">
+        <v>2389</v>
+      </c>
+      <c r="O8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -7810,7 +7901,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -7839,7 +7930,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -7868,7 +7959,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -7897,7 +7988,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -7926,7 +8017,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -7955,7 +8046,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -7984,7 +8075,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -59859,6 +59950,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="693096a9-4944-4f17-a237-baa32704c33d" xsi:nil="true"/>
@@ -59874,15 +59974,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -60135,20 +60226,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1C4E775-5A85-4F92-83E5-7BF232509951}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A5DCB4F-B6CA-455B-962B-DD135DE76577}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="693096a9-4944-4f17-a237-baa32704c33d"/>
     <ds:schemaRef ds:uri="aa4adefa-4376-4f04-8872-3051dc17ebf8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1C4E775-5A85-4F92-83E5-7BF232509951}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>